<commit_message>
Update project tracker: battlegrounds War Room work + scheduled ingest
Logs the battleground redesign (swing gauge, roster, tracking, electorate news,
all-72 rollout, Auckland Central slug fix) and the 4x-daily news/video ingest
schedule to the tracker.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Aratika-Project-Tracker-NEW.xlsx
+++ b/Aratika-Project-Tracker-NEW.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tracker'!$A$1:$F$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tracker'!$A$1:$F$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -651,7 +651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>NEXT_PUBLIC_SUPABASE_URL, SUPABASE_SERVICE_ROLE_KEY, LEGISLATION_RSS_URLS</t>
+          <t>Secrets already configured; added a 2nd workflow (ingest-news.yml) for news/video, 4x daily</t>
         </is>
       </c>
     </row>
@@ -3010,8 +3010,278 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Battlegrounds</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>War Room redesign — dark hero, live election countdown, real swing-to-flip gauge (majority/2, scaled by margin tier)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Replaces old static layout; /battlegrounds/[electorate]</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Battlegrounds</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Roster accordion — tap-to-expand incumbent + confirmed challenger dossiers</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Condensed page; real bio/legislative activity/written Qs per MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Battlegrounds</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Track button — battlegrounds wired into Command Centre bookmarks</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Reused existing 'electorate' bookmark kind, no new infra needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Battlegrounds</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Electorate news/video tagging (Stage 1) — 20 closest 2023 races, by seat + incumbent name</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Real per-candidate tagging deferred until 2026 candidates confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Battlegrounds</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>All-72-electorate rollout — hub lists/filters every seat, not just marginal ones</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Verified via full prod build (283 pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Battlegrounds</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Fixed incumbent-profile slug bug (Auckland Central / Chlöe Swarbrick)</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Real slug was "chle-swarbrick"; page was silently showing zero MP depth</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Editorial / Pipeline</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Scheduled news/video ingest 4x daily (8am/12pm/4pm/7pm NZ)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>New workflow ingest-news.yml; GH Actions cron has no DST awareness — will drift 1hr in NZDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Battlegrounds</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Per-candidate poll % on battle pages</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Shelved — no real NZ electorate-level horse-race polling exists to source honestly</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>MP profile gaps flagged (not fabricated) — missing bio / portfolios / committees</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Collins (Papakura, no bio), Brewer (Upper Harbour), Butterick (Wairarapa), Maipi-Clarke (Hauraki-Waikato), Swarbrick (Auckland Central) — all missing portfolios/committees</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F47"/>
+  <autoFilter ref="A1:F91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>